<commit_message>
fix: relax CPU spec in design/DM/freelancing labs
</commit_message>
<xml_diff>
--- a/lab-standards/BASIS-lab-standard.xlsx
+++ b/lab-standards/BASIS-lab-standard.xlsx
@@ -519,6 +519,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -541,6 +542,7 @@
         <v>25</v>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -583,6 +585,8 @@
       <c r="F8" s="11" t="n"/>
       <c r="G8" s="12" t="n"/>
     </row>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -590,6 +594,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="115.65" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
@@ -601,6 +606,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="26.85" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
@@ -670,7 +676,7 @@
       <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Computers/Laptop: 
-(Minimum Intel Core i5 processor, 8GB RAM (16GB preferred), 500GB SSD storage (1TB preferred), High-resolution monitors (24-inch minimum, with color accuracy).</t>
+(Minimum Intel core i5 or Intel core i3 6 gen/above, or AMD similar spec, 8GB RAM (16GB preferred), 500GB SSD storage (1TB preferred), High-resolution monitors (24-inch minimum, with color accuracy).</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">

</xml_diff>

<commit_message>
fix: revert BASIS UI/UX CPU spec
</commit_message>
<xml_diff>
--- a/lab-standards/BASIS-lab-standard.xlsx
+++ b/lab-standards/BASIS-lab-standard.xlsx
@@ -519,7 +519,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -542,7 +541,6 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -585,8 +583,6 @@
       <c r="F8" s="11" t="n"/>
       <c r="G8" s="12" t="n"/>
     </row>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -594,7 +590,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="115.65" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
@@ -606,7 +601,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="26.85" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
@@ -676,7 +670,7 @@
       <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Computers/Laptop: 
-(Minimum Intel core i5 or Intel core i3 6 gen/above, or AMD Ryzen similar spec, 8GB RAM (16GB preferred), 500GB SSD storage (1TB preferred), High-resolution monitors (24-inch minimum, with color accuracy).</t>
+(Minimum Intel Core i5 processor, 8GB RAM (16GB preferred), 500GB SSD storage (1TB preferred), High-resolution monitors (24-inch minimum, with color accuracy).</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">

</xml_diff>